<commit_message>
Alinha M1/M2 com o ZIP submetido e arruma ficheiros do Sprint 04
- repõe os 3 xlsx de M2 alterados a 13/10 (versão do ZIP)
- retira ficheiros que não estavam no ZIP (m2-readme, xlsx de backlog/sprint backlog M2, cópia duplicada da ata M2)
- move o Sprint Backlog S04 (xlsx) para 01.04 e retira o PDF antigo de 01.06
- retira a cópia duplicada do mapa de pontuação S03 em 01.04

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/01-artefactos-de-gestao/01.06-avaliacao-interna-do-grupo/m2-grelha-rotacao-papeis-v01.xlsx
+++ b/01-artefactos-de-gestao/01.06-avaliacao-interna-do-grupo/m2-grelha-rotacao-papeis-v01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ipppt.sharepoint.com/teams/LEI-GrupodeLDS-UTPORTO/Documentos Partilhados/projeto/01-artefactos-de-gestao/01.06-avaliacao-interna-do-grupo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ipppt.sharepoint.com/teams/LEI-GrupodeLDS-UTPORTO/Documentos Partilhados/Para M2/Gestão/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="463" documentId="13_ncr:1_{F569A737-370C-4B47-9829-76A920C9C4CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84D6EB85-7240-4CD5-9765-1F028A52A886}"/>
+  <xr:revisionPtr revIDLastSave="462" documentId="13_ncr:1_{F569A737-370C-4B47-9829-76A920C9C4CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8199D2C6-2D30-4150-8FDD-99895B57F3A4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Grelha de Rotação de Papéis" sheetId="1" r:id="rId1"/>
@@ -1438,39 +1438,6 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1478,9 +1445,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1501,7 +1465,46 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1513,14 +1516,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1854,68 +1854,68 @@
     <tabColor rgb="FF17365D"/>
   </sheetPr>
   <dimension ref="A1:I60"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="25.375" customWidth="1"/>
-    <col min="2" max="2" width="23.75" customWidth="1"/>
+    <col min="1" max="1" width="25.3984375" customWidth="1"/>
+    <col min="2" max="2" width="23.69921875" customWidth="1"/>
     <col min="3" max="9" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26.1" customHeight="1">
-      <c r="A1" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="I1" s="46" t="s">
+      <c r="A1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="42" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="38.1" customHeight="1">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="D2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="E2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="F2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="28" t="s">
+      <c r="G2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="H2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="29" t="s">
+      <c r="I2" s="40" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1930,94 +1930,94 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:9" ht="21.95" customHeight="1">
-      <c r="A4" s="30" t="s">
+    <row r="4" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A4" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="31" t="s">
+      <c r="C4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="31" t="s">
+      <c r="E4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="31" t="s">
+      <c r="F4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="31" t="s">
+      <c r="G4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="31" t="s">
+      <c r="H4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="I4" s="32" t="s">
+      <c r="I4" s="37" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="24">
+    <row r="5" spans="1:9">
       <c r="A5" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="47">
+      <c r="B5" s="48">
         <v>4</v>
       </c>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="49"/>
-    </row>
-    <row r="6" spans="1:9" ht="24">
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="50"/>
+    </row>
+    <row r="6" spans="1:9" ht="22.8">
       <c r="A6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="52"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="46"/>
+      <c r="I6" s="47"/>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="51"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
-      <c r="G7" s="51"/>
-      <c r="H7" s="51"/>
-      <c r="I7" s="52"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="46"/>
+      <c r="H7" s="46"/>
+      <c r="I7" s="47"/>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="50" t="s">
+      <c r="B8" s="45" t="s">
         <v>262</v>
       </c>
-      <c r="C8" s="51"/>
-      <c r="D8" s="51"/>
-      <c r="E8" s="51"/>
-      <c r="F8" s="51"/>
-      <c r="G8" s="51"/>
-      <c r="H8" s="51"/>
-      <c r="I8" s="52"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="46"/>
+      <c r="I8" s="47"/>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="1"/>
@@ -2030,32 +2030,32 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:9" ht="21.95" customHeight="1">
-      <c r="A10" s="30" t="s">
+    <row r="10" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A10" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="31" t="s">
+      <c r="C10" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="31" t="s">
+      <c r="D10" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="31" t="s">
+      <c r="E10" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="31" t="s">
+      <c r="F10" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="G10" s="31" t="s">
+      <c r="G10" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="H10" s="31" t="s">
+      <c r="H10" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="I10" s="32" t="s">
+      <c r="I10" s="37" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="13.15" customHeight="1">
+    <row r="13" spans="1:9" ht="13.2" customHeight="1">
       <c r="A13" s="6" t="str">
         <f>IF('Listas de apoio'!A6="","",'Listas de apoio'!A6)</f>
         <v>Gonçalo Dinis Magalhães Teixeira</v>
@@ -2251,20 +2251,20 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:9" ht="21.95" customHeight="1">
-      <c r="A17" s="30" t="s">
+    <row r="17" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A17" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="31" t="s">
+      <c r="B17" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="31" t="s">
+      <c r="C17" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="D17" s="31" t="s">
+      <c r="D17" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="32" t="s">
+      <c r="E17" s="37" t="s">
         <v>19</v>
       </c>
       <c r="F17" s="1"/>
@@ -2404,32 +2404,32 @@
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
     </row>
-    <row r="24" spans="1:9" ht="21.95" customHeight="1">
-      <c r="A24" s="30" t="s">
+    <row r="24" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A24" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="31" t="s">
+      <c r="C24" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="D24" s="31" t="s">
+      <c r="D24" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="E24" s="31" t="s">
+      <c r="E24" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="F24" s="31" t="s">
+      <c r="F24" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="32" t="s">
+      <c r="G24" s="37" t="s">
         <v>29</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
     </row>
-    <row r="25" spans="1:9" ht="39.950000000000003" customHeight="1">
+    <row r="25" spans="1:9" ht="39.9" customHeight="1">
       <c r="A25" s="5" t="s">
         <v>30</v>
       </c>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="G30" s="6" t="str">
         <f>IF(B30="","",IF(COUNTIFS('Registo da Rotação'!$A$6:$A$25,A30,'Registo da Rotação'!$D$6:$D$25,"Em curso")&gt;0,"Em avaliação",IF(COUNTIFS('Registo da Rotação'!$A$6:$A$25,A30,'Registo da Rotação'!$D$6:$D$25,"Concluído")=0,"Sem sprints concluídos",IF(COUNTIF('Registo da Rotação'!$B$54:$B$162,A30)&lt;$B$5,"Não aplicável — tarefas insuficientes",IF(AND(C30&gt;0,D30&gt;0,E30&gt;0),"Cumprida","Por cumprir")))))</f>
-        <v>Cumprida</v>
+        <v>Em avaliação</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="G31" s="6" t="str">
         <f>IF(B31="","",IF(COUNTIFS('Registo da Rotação'!$A$6:$A$25,A31,'Registo da Rotação'!$D$6:$D$25,"Em curso")&gt;0,"Em avaliação",IF(COUNTIFS('Registo da Rotação'!$A$6:$A$25,A31,'Registo da Rotação'!$D$6:$D$25,"Concluído")=0,"Sem sprints concluídos",IF(COUNTIF('Registo da Rotação'!$B$54:$B$162,A31)&lt;$B$5,"Não aplicável — tarefas insuficientes",IF(AND(C31&gt;0,D31&gt;0,E31&gt;0),"Cumprida","Por cumprir")))))</f>
-        <v>Cumprida</v>
+        <v>Em avaliação</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
@@ -2673,7 +2673,7 @@
       </c>
       <c r="G32" s="6" t="str">
         <f>IF(B32="","",IF(COUNTIFS('Registo da Rotação'!$A$6:$A$25,A32,'Registo da Rotação'!$D$6:$D$25,"Em curso")&gt;0,"Em avaliação",IF(COUNTIFS('Registo da Rotação'!$A$6:$A$25,A32,'Registo da Rotação'!$D$6:$D$25,"Concluído")=0,"Sem sprints concluídos",IF(COUNTIF('Registo da Rotação'!$B$54:$B$162,A32)&lt;$B$5,"Não aplicável — tarefas insuficientes",IF(AND(C32&gt;0,D32&gt;0,E32&gt;0),"Cumprida","Por cumprir")))))</f>
-        <v>Cumprida</v>
+        <v>Em avaliação</v>
       </c>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
@@ -2705,7 +2705,7 @@
       </c>
       <c r="G33" s="6" t="str">
         <f>IF(B33="","",IF(COUNTIFS('Registo da Rotação'!$A$6:$A$25,A33,'Registo da Rotação'!$D$6:$D$25,"Em curso")&gt;0,"Em avaliação",IF(COUNTIFS('Registo da Rotação'!$A$6:$A$25,A33,'Registo da Rotação'!$D$6:$D$25,"Concluído")=0,"Sem sprints concluídos",IF(COUNTIF('Registo da Rotação'!$B$54:$B$162,A33)&lt;$B$5,"Não aplicável — tarefas insuficientes",IF(AND(C33&gt;0,D33&gt;0,E33&gt;0),"Cumprida","Por cumprir")))))</f>
-        <v>Cumprida</v>
+        <v>Em avaliação</v>
       </c>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
@@ -3177,16 +3177,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B6:I6"/>
     <mergeCell ref="B7:I7"/>
     <mergeCell ref="B8:I8"/>
     <mergeCell ref="A10:I10"/>
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B6:I6"/>
   </mergeCells>
   <conditionalFormatting sqref="E19:E22">
     <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Rever"/>
@@ -3215,101 +3215,101 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R219"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="10.125" customWidth="1"/>
+    <col min="2" max="2" width="10.09765625" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="24.125" customWidth="1"/>
-    <col min="7" max="7" width="18.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.25" customWidth="1"/>
+    <col min="6" max="6" width="24.09765625" customWidth="1"/>
+    <col min="7" max="7" width="18.09765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.296875" customWidth="1"/>
     <col min="9" max="9" width="9.5" customWidth="1"/>
-    <col min="10" max="10" width="5.875" customWidth="1"/>
+    <col min="10" max="10" width="5.8984375" customWidth="1"/>
     <col min="11" max="11" width="17" customWidth="1"/>
-    <col min="12" max="12" width="10.625" customWidth="1"/>
-    <col min="13" max="13" width="10.125" customWidth="1"/>
-    <col min="14" max="14" width="24.75" customWidth="1"/>
-    <col min="15" max="17" width="12.625" customWidth="1"/>
+    <col min="12" max="12" width="10.59765625" customWidth="1"/>
+    <col min="13" max="13" width="10.09765625" customWidth="1"/>
+    <col min="14" max="14" width="24.796875" customWidth="1"/>
+    <col min="15" max="17" width="12.59765625" customWidth="1"/>
     <col min="18" max="18" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="26.1" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
+      <c r="K1" s="52"/>
+      <c r="L1" s="52"/>
+      <c r="M1" s="52"/>
+      <c r="N1" s="52"/>
+      <c r="O1" s="52"/>
+      <c r="P1" s="52"/>
+      <c r="Q1" s="52"/>
+      <c r="R1" s="52"/>
     </row>
     <row r="2" spans="1:18" ht="38.1" customHeight="1">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="D2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="E2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="F2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="28" t="s">
+      <c r="G2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="H2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="28" t="s">
+      <c r="I2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="J2" s="28" t="s">
+      <c r="J2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="K2" s="28" t="s">
+      <c r="K2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="L2" s="28" t="s">
+      <c r="L2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="M2" s="28" t="s">
+      <c r="M2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="N2" s="28" t="s">
+      <c r="N2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="O2" s="28" t="s">
+      <c r="O2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="P2" s="28" t="s">
+      <c r="P2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="Q2" s="28" t="s">
+      <c r="Q2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="R2" s="29" t="s">
+      <c r="R2" s="40" t="s">
         <v>36</v>
       </c>
     </row>
@@ -3333,26 +3333,26 @@
       <c r="Q3" s="1"/>
       <c r="R3" s="1"/>
     </row>
-    <row r="4" spans="1:18" ht="21.95" customHeight="1">
-      <c r="A4" s="30" t="s">
+    <row r="4" spans="1:18" ht="21.9" customHeight="1">
+      <c r="A4" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="31" t="s">
+      <c r="C4" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="31" t="s">
+      <c r="E4" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="31" t="s">
+      <c r="F4" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="32" t="s">
+      <c r="G4" s="37" t="s">
         <v>37</v>
       </c>
       <c r="H4" s="1"/>
@@ -3367,7 +3367,7 @@
       <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
     </row>
-    <row r="5" spans="1:18" ht="33.75">
+    <row r="5" spans="1:18" ht="20.399999999999999">
       <c r="A5" s="5" t="s">
         <v>30</v>
       </c>
@@ -3401,7 +3401,7 @@
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
     </row>
-    <row r="6" spans="1:18" ht="24">
+    <row r="6" spans="1:18">
       <c r="A6" s="3" t="s">
         <v>215</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>219</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>46</v>
+        <v>217</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>262</v>
@@ -3849,59 +3849,59 @@
       <c r="Q26" s="1"/>
       <c r="R26" s="1"/>
     </row>
-    <row r="27" spans="1:18" ht="21.95" customHeight="1">
-      <c r="A27" s="30" t="s">
+    <row r="27" spans="1:18" ht="21.9" customHeight="1">
+      <c r="A27" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="C27" s="31" t="s">
+      <c r="C27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="D27" s="31" t="s">
+      <c r="D27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="E27" s="31" t="s">
+      <c r="E27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="F27" s="31" t="s">
+      <c r="F27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="G27" s="31" t="s">
+      <c r="G27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="H27" s="31" t="s">
+      <c r="H27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="I27" s="31" t="s">
+      <c r="I27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="J27" s="31" t="s">
+      <c r="J27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="K27" s="31" t="s">
+      <c r="K27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="L27" s="31" t="s">
+      <c r="L27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="M27" s="31" t="s">
+      <c r="M27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="N27" s="31" t="s">
+      <c r="N27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="O27" s="31" t="s">
+      <c r="O27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="P27" s="31" t="s">
+      <c r="P27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="Q27" s="31" t="s">
+      <c r="Q27" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="R27" s="32" t="s">
+      <c r="R27" s="37" t="s">
         <v>50</v>
       </c>
     </row>
@@ -3912,30 +3912,30 @@
       <c r="B28" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="33" t="s">
+      <c r="C28" s="44" t="s">
         <v>248</v>
       </c>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33" t="s">
+      <c r="D28" s="44"/>
+      <c r="E28" s="44"/>
+      <c r="F28" s="44"/>
+      <c r="G28" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="33"/>
-      <c r="K28" s="33" t="s">
+      <c r="H28" s="44"/>
+      <c r="I28" s="44"/>
+      <c r="J28" s="44"/>
+      <c r="K28" s="44" t="s">
         <v>249</v>
       </c>
-      <c r="L28" s="33"/>
-      <c r="M28" s="33"/>
-      <c r="N28" s="33"/>
-      <c r="O28" s="33" t="s">
+      <c r="L28" s="44"/>
+      <c r="M28" s="44"/>
+      <c r="N28" s="44"/>
+      <c r="O28" s="44" t="s">
         <v>52</v>
       </c>
-      <c r="P28" s="33"/>
-      <c r="Q28" s="33"/>
-      <c r="R28" s="33"/>
+      <c r="P28" s="44"/>
+      <c r="Q28" s="44"/>
+      <c r="R28" s="44"/>
     </row>
     <row r="29" spans="1:18" ht="32.1" customHeight="1">
       <c r="A29" s="3" t="s">
@@ -3944,30 +3944,30 @@
       <c r="B29" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="C29" s="34" t="s">
+      <c r="C29" s="41" t="s">
         <v>263</v>
       </c>
-      <c r="D29" s="35"/>
-      <c r="E29" s="35"/>
-      <c r="F29" s="35"/>
-      <c r="G29" s="34" t="s">
+      <c r="D29" s="34"/>
+      <c r="E29" s="34"/>
+      <c r="F29" s="34"/>
+      <c r="G29" s="41" t="s">
         <v>264</v>
       </c>
-      <c r="H29" s="35"/>
-      <c r="I29" s="35"/>
-      <c r="J29" s="35"/>
-      <c r="K29" s="34" t="s">
+      <c r="H29" s="34"/>
+      <c r="I29" s="34"/>
+      <c r="J29" s="34"/>
+      <c r="K29" s="41" t="s">
         <v>285</v>
       </c>
-      <c r="L29" s="35"/>
-      <c r="M29" s="35"/>
-      <c r="N29" s="35"/>
-      <c r="O29" s="34" t="s">
+      <c r="L29" s="34"/>
+      <c r="M29" s="34"/>
+      <c r="N29" s="34"/>
+      <c r="O29" s="41" t="s">
         <v>286</v>
       </c>
-      <c r="P29" s="35"/>
-      <c r="Q29" s="35"/>
-      <c r="R29" s="35"/>
+      <c r="P29" s="34"/>
+      <c r="Q29" s="34"/>
+      <c r="R29" s="34"/>
     </row>
     <row r="30" spans="1:18" ht="32.1" customHeight="1">
       <c r="A30" s="3" t="s">
@@ -3976,390 +3976,390 @@
       <c r="B30" s="24" t="s">
         <v>217</v>
       </c>
-      <c r="C30" s="35" t="s">
+      <c r="C30" s="34" t="s">
         <v>313</v>
       </c>
-      <c r="D30" s="35"/>
-      <c r="E30" s="35"/>
-      <c r="F30" s="35"/>
-      <c r="G30" s="35" t="s">
+      <c r="D30" s="34"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="34" t="s">
         <v>314</v>
       </c>
-      <c r="H30" s="35"/>
-      <c r="I30" s="35"/>
-      <c r="J30" s="35"/>
-      <c r="K30" s="35" t="s">
+      <c r="H30" s="34"/>
+      <c r="I30" s="34"/>
+      <c r="J30" s="34"/>
+      <c r="K30" s="34" t="s">
         <v>315</v>
       </c>
-      <c r="L30" s="35"/>
-      <c r="M30" s="35"/>
-      <c r="N30" s="35"/>
-      <c r="O30" s="35" t="s">
+      <c r="L30" s="34"/>
+      <c r="M30" s="34"/>
+      <c r="N30" s="34"/>
+      <c r="O30" s="34" t="s">
         <v>316</v>
       </c>
-      <c r="P30" s="35"/>
-      <c r="Q30" s="35"/>
-      <c r="R30" s="35"/>
+      <c r="P30" s="34"/>
+      <c r="Q30" s="34"/>
+      <c r="R30" s="34"/>
     </row>
     <row r="31" spans="1:18" ht="32.1" customHeight="1">
       <c r="A31" s="3"/>
       <c r="B31" s="24"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="35"/>
-      <c r="E31" s="35"/>
-      <c r="F31" s="35"/>
-      <c r="G31" s="35"/>
-      <c r="H31" s="35"/>
-      <c r="I31" s="35"/>
-      <c r="J31" s="35"/>
-      <c r="K31" s="35"/>
-      <c r="L31" s="35"/>
-      <c r="M31" s="35"/>
-      <c r="N31" s="35"/>
-      <c r="O31" s="35"/>
-      <c r="P31" s="35"/>
-      <c r="Q31" s="35"/>
-      <c r="R31" s="35"/>
+      <c r="C31" s="34"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="34"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="34"/>
+      <c r="I31" s="34"/>
+      <c r="J31" s="34"/>
+      <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
+      <c r="M31" s="34"/>
+      <c r="N31" s="34"/>
+      <c r="O31" s="34"/>
+      <c r="P31" s="34"/>
+      <c r="Q31" s="34"/>
+      <c r="R31" s="34"/>
     </row>
     <row r="32" spans="1:18" ht="32.1" customHeight="1">
       <c r="A32" s="3"/>
       <c r="B32" s="24"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="37"/>
-      <c r="E32" s="37"/>
-      <c r="F32" s="38"/>
-      <c r="G32" s="36"/>
-      <c r="H32" s="37"/>
-      <c r="I32" s="37"/>
-      <c r="J32" s="38"/>
-      <c r="K32" s="36"/>
-      <c r="L32" s="37"/>
-      <c r="M32" s="37"/>
-      <c r="N32" s="38"/>
-      <c r="O32" s="36"/>
-      <c r="P32" s="37"/>
-      <c r="Q32" s="37"/>
-      <c r="R32" s="38"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="26"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="25"/>
+      <c r="L32" s="26"/>
+      <c r="M32" s="26"/>
+      <c r="N32" s="27"/>
+      <c r="O32" s="25"/>
+      <c r="P32" s="26"/>
+      <c r="Q32" s="26"/>
+      <c r="R32" s="27"/>
     </row>
     <row r="33" spans="1:18" ht="32.1" customHeight="1">
       <c r="A33" s="3"/>
       <c r="B33" s="24"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="35"/>
-      <c r="J33" s="35"/>
-      <c r="K33" s="35"/>
-      <c r="L33" s="35"/>
-      <c r="M33" s="35"/>
-      <c r="N33" s="35"/>
-      <c r="O33" s="35"/>
-      <c r="P33" s="35"/>
-      <c r="Q33" s="35"/>
-      <c r="R33" s="35"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="34"/>
+      <c r="I33" s="34"/>
+      <c r="J33" s="34"/>
+      <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
+      <c r="M33" s="34"/>
+      <c r="N33" s="34"/>
+      <c r="O33" s="34"/>
+      <c r="P33" s="34"/>
+      <c r="Q33" s="34"/>
+      <c r="R33" s="34"/>
     </row>
     <row r="34" spans="1:18" ht="32.1" customHeight="1">
       <c r="A34" s="3"/>
       <c r="B34" s="24"/>
-      <c r="C34" s="36"/>
-      <c r="D34" s="37"/>
-      <c r="E34" s="37"/>
-      <c r="F34" s="38"/>
-      <c r="G34" s="36"/>
-      <c r="H34" s="37"/>
-      <c r="I34" s="37"/>
-      <c r="J34" s="38"/>
-      <c r="K34" s="36"/>
-      <c r="L34" s="37"/>
-      <c r="M34" s="37"/>
-      <c r="N34" s="38"/>
-      <c r="O34" s="36"/>
-      <c r="P34" s="37"/>
-      <c r="Q34" s="37"/>
-      <c r="R34" s="38"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="26"/>
+      <c r="I34" s="26"/>
+      <c r="J34" s="27"/>
+      <c r="K34" s="25"/>
+      <c r="L34" s="26"/>
+      <c r="M34" s="26"/>
+      <c r="N34" s="27"/>
+      <c r="O34" s="25"/>
+      <c r="P34" s="26"/>
+      <c r="Q34" s="26"/>
+      <c r="R34" s="27"/>
     </row>
     <row r="35" spans="1:18" ht="32.1" customHeight="1">
       <c r="A35" s="3"/>
       <c r="B35" s="24"/>
-      <c r="C35" s="36"/>
-      <c r="D35" s="37"/>
-      <c r="E35" s="37"/>
-      <c r="F35" s="38"/>
-      <c r="G35" s="36"/>
-      <c r="H35" s="37"/>
-      <c r="I35" s="37"/>
-      <c r="J35" s="38"/>
-      <c r="K35" s="36"/>
-      <c r="L35" s="37"/>
-      <c r="M35" s="37"/>
-      <c r="N35" s="38"/>
-      <c r="O35" s="36"/>
-      <c r="P35" s="37"/>
-      <c r="Q35" s="37"/>
-      <c r="R35" s="38"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="25"/>
+      <c r="H35" s="26"/>
+      <c r="I35" s="26"/>
+      <c r="J35" s="27"/>
+      <c r="K35" s="25"/>
+      <c r="L35" s="26"/>
+      <c r="M35" s="26"/>
+      <c r="N35" s="27"/>
+      <c r="O35" s="25"/>
+      <c r="P35" s="26"/>
+      <c r="Q35" s="26"/>
+      <c r="R35" s="27"/>
     </row>
     <row r="36" spans="1:18" ht="32.1" customHeight="1">
       <c r="A36" s="3"/>
       <c r="B36" s="24"/>
-      <c r="C36" s="36"/>
-      <c r="D36" s="37"/>
-      <c r="E36" s="37"/>
-      <c r="F36" s="38"/>
-      <c r="G36" s="36"/>
-      <c r="H36" s="37"/>
-      <c r="I36" s="37"/>
-      <c r="J36" s="38"/>
-      <c r="K36" s="36"/>
-      <c r="L36" s="37"/>
-      <c r="M36" s="37"/>
-      <c r="N36" s="38"/>
-      <c r="O36" s="36"/>
-      <c r="P36" s="37"/>
-      <c r="Q36" s="37"/>
-      <c r="R36" s="38"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="27"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="26"/>
+      <c r="J36" s="27"/>
+      <c r="K36" s="25"/>
+      <c r="L36" s="26"/>
+      <c r="M36" s="26"/>
+      <c r="N36" s="27"/>
+      <c r="O36" s="25"/>
+      <c r="P36" s="26"/>
+      <c r="Q36" s="26"/>
+      <c r="R36" s="27"/>
     </row>
     <row r="37" spans="1:18" ht="32.1" customHeight="1">
       <c r="A37" s="3"/>
       <c r="B37" s="24"/>
-      <c r="C37" s="36"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="37"/>
-      <c r="F37" s="38"/>
-      <c r="G37" s="36"/>
-      <c r="H37" s="37"/>
-      <c r="I37" s="37"/>
-      <c r="J37" s="38"/>
-      <c r="K37" s="36"/>
-      <c r="L37" s="37"/>
-      <c r="M37" s="37"/>
-      <c r="N37" s="38"/>
-      <c r="O37" s="36"/>
-      <c r="P37" s="37"/>
-      <c r="Q37" s="37"/>
-      <c r="R37" s="38"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="26"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="26"/>
+      <c r="I37" s="26"/>
+      <c r="J37" s="27"/>
+      <c r="K37" s="25"/>
+      <c r="L37" s="26"/>
+      <c r="M37" s="26"/>
+      <c r="N37" s="27"/>
+      <c r="O37" s="25"/>
+      <c r="P37" s="26"/>
+      <c r="Q37" s="26"/>
+      <c r="R37" s="27"/>
     </row>
     <row r="38" spans="1:18" ht="32.1" customHeight="1">
       <c r="A38" s="3"/>
       <c r="B38" s="24"/>
-      <c r="C38" s="36"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="37"/>
-      <c r="F38" s="38"/>
-      <c r="G38" s="36"/>
-      <c r="H38" s="37"/>
-      <c r="I38" s="37"/>
-      <c r="J38" s="38"/>
-      <c r="K38" s="36"/>
-      <c r="L38" s="37"/>
-      <c r="M38" s="37"/>
-      <c r="N38" s="38"/>
-      <c r="O38" s="36"/>
-      <c r="P38" s="37"/>
-      <c r="Q38" s="37"/>
-      <c r="R38" s="38"/>
+      <c r="C38" s="25"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="26"/>
+      <c r="F38" s="27"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="26"/>
+      <c r="I38" s="26"/>
+      <c r="J38" s="27"/>
+      <c r="K38" s="25"/>
+      <c r="L38" s="26"/>
+      <c r="M38" s="26"/>
+      <c r="N38" s="27"/>
+      <c r="O38" s="25"/>
+      <c r="P38" s="26"/>
+      <c r="Q38" s="26"/>
+      <c r="R38" s="27"/>
     </row>
     <row r="39" spans="1:18" ht="32.1" customHeight="1">
       <c r="A39" s="3"/>
       <c r="B39" s="24"/>
-      <c r="C39" s="36"/>
-      <c r="D39" s="37"/>
-      <c r="E39" s="37"/>
-      <c r="F39" s="38"/>
-      <c r="G39" s="36"/>
-      <c r="H39" s="37"/>
-      <c r="I39" s="37"/>
-      <c r="J39" s="38"/>
-      <c r="K39" s="36"/>
-      <c r="L39" s="37"/>
-      <c r="M39" s="37"/>
-      <c r="N39" s="38"/>
-      <c r="O39" s="36"/>
-      <c r="P39" s="37"/>
-      <c r="Q39" s="37"/>
-      <c r="R39" s="38"/>
+      <c r="C39" s="25"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="26"/>
+      <c r="F39" s="27"/>
+      <c r="G39" s="25"/>
+      <c r="H39" s="26"/>
+      <c r="I39" s="26"/>
+      <c r="J39" s="27"/>
+      <c r="K39" s="25"/>
+      <c r="L39" s="26"/>
+      <c r="M39" s="26"/>
+      <c r="N39" s="27"/>
+      <c r="O39" s="25"/>
+      <c r="P39" s="26"/>
+      <c r="Q39" s="26"/>
+      <c r="R39" s="27"/>
     </row>
     <row r="40" spans="1:18" ht="32.1" customHeight="1">
       <c r="A40" s="3"/>
       <c r="B40" s="24"/>
-      <c r="C40" s="36"/>
-      <c r="D40" s="37"/>
-      <c r="E40" s="37"/>
-      <c r="F40" s="38"/>
-      <c r="G40" s="36"/>
-      <c r="H40" s="37"/>
-      <c r="I40" s="37"/>
-      <c r="J40" s="38"/>
-      <c r="K40" s="36"/>
-      <c r="L40" s="37"/>
-      <c r="M40" s="37"/>
-      <c r="N40" s="38"/>
-      <c r="O40" s="36"/>
-      <c r="P40" s="37"/>
-      <c r="Q40" s="37"/>
-      <c r="R40" s="38"/>
+      <c r="C40" s="25"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="25"/>
+      <c r="H40" s="26"/>
+      <c r="I40" s="26"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="25"/>
+      <c r="L40" s="26"/>
+      <c r="M40" s="26"/>
+      <c r="N40" s="27"/>
+      <c r="O40" s="25"/>
+      <c r="P40" s="26"/>
+      <c r="Q40" s="26"/>
+      <c r="R40" s="27"/>
     </row>
     <row r="41" spans="1:18" ht="32.1" customHeight="1">
       <c r="A41" s="3"/>
       <c r="B41" s="24"/>
-      <c r="C41" s="36"/>
-      <c r="D41" s="37"/>
-      <c r="E41" s="37"/>
-      <c r="F41" s="38"/>
-      <c r="G41" s="36"/>
-      <c r="H41" s="37"/>
-      <c r="I41" s="37"/>
-      <c r="J41" s="38"/>
-      <c r="K41" s="36"/>
-      <c r="L41" s="37"/>
-      <c r="M41" s="37"/>
-      <c r="N41" s="38"/>
-      <c r="O41" s="36"/>
-      <c r="P41" s="37"/>
-      <c r="Q41" s="37"/>
-      <c r="R41" s="38"/>
+      <c r="C41" s="25"/>
+      <c r="D41" s="26"/>
+      <c r="E41" s="26"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="25"/>
+      <c r="H41" s="26"/>
+      <c r="I41" s="26"/>
+      <c r="J41" s="27"/>
+      <c r="K41" s="25"/>
+      <c r="L41" s="26"/>
+      <c r="M41" s="26"/>
+      <c r="N41" s="27"/>
+      <c r="O41" s="25"/>
+      <c r="P41" s="26"/>
+      <c r="Q41" s="26"/>
+      <c r="R41" s="27"/>
     </row>
     <row r="42" spans="1:18" ht="32.1" customHeight="1">
       <c r="A42" s="3"/>
       <c r="B42" s="24"/>
-      <c r="C42" s="36"/>
-      <c r="D42" s="37"/>
-      <c r="E42" s="37"/>
-      <c r="F42" s="38"/>
-      <c r="G42" s="36"/>
-      <c r="H42" s="37"/>
-      <c r="I42" s="37"/>
-      <c r="J42" s="38"/>
-      <c r="K42" s="36"/>
-      <c r="L42" s="37"/>
-      <c r="M42" s="37"/>
-      <c r="N42" s="38"/>
-      <c r="O42" s="36"/>
-      <c r="P42" s="37"/>
-      <c r="Q42" s="37"/>
-      <c r="R42" s="38"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="26"/>
+      <c r="E42" s="26"/>
+      <c r="F42" s="27"/>
+      <c r="G42" s="25"/>
+      <c r="H42" s="26"/>
+      <c r="I42" s="26"/>
+      <c r="J42" s="27"/>
+      <c r="K42" s="25"/>
+      <c r="L42" s="26"/>
+      <c r="M42" s="26"/>
+      <c r="N42" s="27"/>
+      <c r="O42" s="25"/>
+      <c r="P42" s="26"/>
+      <c r="Q42" s="26"/>
+      <c r="R42" s="27"/>
     </row>
     <row r="43" spans="1:18" ht="32.1" customHeight="1">
       <c r="A43" s="3"/>
       <c r="B43" s="24"/>
-      <c r="C43" s="36"/>
-      <c r="D43" s="37"/>
-      <c r="E43" s="37"/>
-      <c r="F43" s="38"/>
-      <c r="G43" s="36"/>
-      <c r="H43" s="37"/>
-      <c r="I43" s="37"/>
-      <c r="J43" s="38"/>
-      <c r="K43" s="36"/>
-      <c r="L43" s="37"/>
-      <c r="M43" s="37"/>
-      <c r="N43" s="38"/>
-      <c r="O43" s="36"/>
-      <c r="P43" s="37"/>
-      <c r="Q43" s="37"/>
-      <c r="R43" s="38"/>
+      <c r="C43" s="25"/>
+      <c r="D43" s="26"/>
+      <c r="E43" s="26"/>
+      <c r="F43" s="27"/>
+      <c r="G43" s="25"/>
+      <c r="H43" s="26"/>
+      <c r="I43" s="26"/>
+      <c r="J43" s="27"/>
+      <c r="K43" s="25"/>
+      <c r="L43" s="26"/>
+      <c r="M43" s="26"/>
+      <c r="N43" s="27"/>
+      <c r="O43" s="25"/>
+      <c r="P43" s="26"/>
+      <c r="Q43" s="26"/>
+      <c r="R43" s="27"/>
     </row>
     <row r="44" spans="1:18" ht="32.1" customHeight="1">
       <c r="A44" s="3"/>
       <c r="B44" s="24"/>
-      <c r="C44" s="36"/>
-      <c r="D44" s="37"/>
-      <c r="E44" s="37"/>
-      <c r="F44" s="38"/>
-      <c r="G44" s="36"/>
-      <c r="H44" s="37"/>
-      <c r="I44" s="37"/>
-      <c r="J44" s="38"/>
-      <c r="K44" s="36"/>
-      <c r="L44" s="37"/>
-      <c r="M44" s="37"/>
-      <c r="N44" s="38"/>
-      <c r="O44" s="36"/>
-      <c r="P44" s="37"/>
-      <c r="Q44" s="37"/>
-      <c r="R44" s="38"/>
+      <c r="C44" s="25"/>
+      <c r="D44" s="26"/>
+      <c r="E44" s="26"/>
+      <c r="F44" s="27"/>
+      <c r="G44" s="25"/>
+      <c r="H44" s="26"/>
+      <c r="I44" s="26"/>
+      <c r="J44" s="27"/>
+      <c r="K44" s="25"/>
+      <c r="L44" s="26"/>
+      <c r="M44" s="26"/>
+      <c r="N44" s="27"/>
+      <c r="O44" s="25"/>
+      <c r="P44" s="26"/>
+      <c r="Q44" s="26"/>
+      <c r="R44" s="27"/>
     </row>
     <row r="45" spans="1:18" ht="32.1" customHeight="1">
       <c r="A45" s="3"/>
       <c r="B45" s="24"/>
-      <c r="C45" s="36"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="37"/>
-      <c r="F45" s="38"/>
-      <c r="G45" s="36"/>
-      <c r="H45" s="37"/>
-      <c r="I45" s="37"/>
-      <c r="J45" s="38"/>
-      <c r="K45" s="36"/>
-      <c r="L45" s="37"/>
-      <c r="M45" s="37"/>
-      <c r="N45" s="38"/>
-      <c r="O45" s="36"/>
-      <c r="P45" s="37"/>
-      <c r="Q45" s="37"/>
-      <c r="R45" s="38"/>
+      <c r="C45" s="25"/>
+      <c r="D45" s="26"/>
+      <c r="E45" s="26"/>
+      <c r="F45" s="27"/>
+      <c r="G45" s="25"/>
+      <c r="H45" s="26"/>
+      <c r="I45" s="26"/>
+      <c r="J45" s="27"/>
+      <c r="K45" s="25"/>
+      <c r="L45" s="26"/>
+      <c r="M45" s="26"/>
+      <c r="N45" s="27"/>
+      <c r="O45" s="25"/>
+      <c r="P45" s="26"/>
+      <c r="Q45" s="26"/>
+      <c r="R45" s="27"/>
     </row>
     <row r="46" spans="1:18" ht="32.1" customHeight="1">
       <c r="A46" s="3"/>
       <c r="B46" s="24"/>
-      <c r="C46" s="36"/>
-      <c r="D46" s="37"/>
-      <c r="E46" s="37"/>
-      <c r="F46" s="38"/>
-      <c r="G46" s="36"/>
-      <c r="H46" s="37"/>
-      <c r="I46" s="37"/>
-      <c r="J46" s="38"/>
-      <c r="K46" s="36"/>
-      <c r="L46" s="37"/>
-      <c r="M46" s="37"/>
-      <c r="N46" s="38"/>
-      <c r="O46" s="36"/>
-      <c r="P46" s="37"/>
-      <c r="Q46" s="37"/>
-      <c r="R46" s="38"/>
+      <c r="C46" s="25"/>
+      <c r="D46" s="26"/>
+      <c r="E46" s="26"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="25"/>
+      <c r="H46" s="26"/>
+      <c r="I46" s="26"/>
+      <c r="J46" s="27"/>
+      <c r="K46" s="25"/>
+      <c r="L46" s="26"/>
+      <c r="M46" s="26"/>
+      <c r="N46" s="27"/>
+      <c r="O46" s="25"/>
+      <c r="P46" s="26"/>
+      <c r="Q46" s="26"/>
+      <c r="R46" s="27"/>
     </row>
     <row r="47" spans="1:18" ht="32.1" customHeight="1">
       <c r="A47" s="3"/>
       <c r="B47" s="24"/>
-      <c r="C47" s="36"/>
-      <c r="D47" s="37"/>
-      <c r="E47" s="37"/>
-      <c r="F47" s="38"/>
-      <c r="G47" s="36"/>
-      <c r="H47" s="37"/>
-      <c r="I47" s="37"/>
-      <c r="J47" s="38"/>
-      <c r="K47" s="36"/>
-      <c r="L47" s="37"/>
-      <c r="M47" s="37"/>
-      <c r="N47" s="38"/>
-      <c r="O47" s="36"/>
-      <c r="P47" s="37"/>
-      <c r="Q47" s="37"/>
-      <c r="R47" s="38"/>
+      <c r="C47" s="25"/>
+      <c r="D47" s="26"/>
+      <c r="E47" s="26"/>
+      <c r="F47" s="27"/>
+      <c r="G47" s="25"/>
+      <c r="H47" s="26"/>
+      <c r="I47" s="26"/>
+      <c r="J47" s="27"/>
+      <c r="K47" s="25"/>
+      <c r="L47" s="26"/>
+      <c r="M47" s="26"/>
+      <c r="N47" s="27"/>
+      <c r="O47" s="25"/>
+      <c r="P47" s="26"/>
+      <c r="Q47" s="26"/>
+      <c r="R47" s="27"/>
     </row>
     <row r="48" spans="1:18" ht="32.1" customHeight="1">
       <c r="A48" s="3"/>
       <c r="B48" s="24"/>
-      <c r="C48" s="35"/>
-      <c r="D48" s="35"/>
-      <c r="E48" s="35"/>
-      <c r="F48" s="35"/>
-      <c r="G48" s="35"/>
-      <c r="H48" s="35"/>
-      <c r="I48" s="35"/>
-      <c r="J48" s="35"/>
-      <c r="K48" s="35"/>
-      <c r="L48" s="35"/>
-      <c r="M48" s="35"/>
-      <c r="N48" s="35"/>
-      <c r="O48" s="35"/>
-      <c r="P48" s="35"/>
-      <c r="Q48" s="35"/>
-      <c r="R48" s="35"/>
+      <c r="C48" s="34"/>
+      <c r="D48" s="34"/>
+      <c r="E48" s="34"/>
+      <c r="F48" s="34"/>
+      <c r="G48" s="34"/>
+      <c r="H48" s="34"/>
+      <c r="I48" s="34"/>
+      <c r="J48" s="34"/>
+      <c r="K48" s="34"/>
+      <c r="L48" s="34"/>
+      <c r="M48" s="34"/>
+      <c r="N48" s="34"/>
+      <c r="O48" s="34"/>
+      <c r="P48" s="34"/>
+      <c r="Q48" s="34"/>
+      <c r="R48" s="34"/>
     </row>
     <row r="49" spans="1:18">
       <c r="A49" s="1"/>
@@ -4401,38 +4401,38 @@
       <c r="Q50" s="1"/>
       <c r="R50" s="1"/>
     </row>
-    <row r="51" spans="1:18" ht="21.95" customHeight="1">
-      <c r="A51" s="30" t="s">
+    <row r="51" spans="1:18" ht="21.9" customHeight="1">
+      <c r="A51" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="B51" s="31" t="s">
+      <c r="B51" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="C51" s="31" t="s">
+      <c r="C51" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="D51" s="31" t="s">
+      <c r="D51" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="E51" s="31" t="s">
+      <c r="E51" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="F51" s="31" t="s">
+      <c r="F51" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="G51" s="31" t="s">
+      <c r="G51" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="H51" s="31" t="s">
+      <c r="H51" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="I51" s="31" t="s">
+      <c r="I51" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="J51" s="31" t="s">
+      <c r="J51" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="K51" s="32" t="s">
+      <c r="K51" s="37" t="s">
         <v>53</v>
       </c>
       <c r="L51" s="1"/>
@@ -4443,38 +4443,38 @@
       <c r="Q51" s="1"/>
       <c r="R51" s="1"/>
     </row>
-    <row r="52" spans="1:18" ht="33.950000000000003" customHeight="1">
-      <c r="A52" s="39" t="s">
+    <row r="52" spans="1:18" ht="33.9" customHeight="1">
+      <c r="A52" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="B52" s="28" t="s">
+      <c r="B52" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="C52" s="28" t="s">
+      <c r="C52" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="D52" s="28" t="s">
+      <c r="D52" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="E52" s="28" t="s">
+      <c r="E52" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="F52" s="28" t="s">
+      <c r="F52" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="G52" s="28" t="s">
+      <c r="G52" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="H52" s="28" t="s">
+      <c r="H52" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="I52" s="28" t="s">
+      <c r="I52" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="J52" s="28" t="s">
+      <c r="J52" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="K52" s="29" t="s">
+      <c r="K52" s="40" t="s">
         <v>54</v>
       </c>
       <c r="L52" s="1"/>
@@ -4485,7 +4485,7 @@
       <c r="Q52" s="1"/>
       <c r="R52" s="1"/>
     </row>
-    <row r="53" spans="1:18" ht="39.950000000000003" customHeight="1">
+    <row r="53" spans="1:18" ht="39.9" customHeight="1">
       <c r="A53" s="5" t="s">
         <v>55</v>
       </c>
@@ -4527,7 +4527,7 @@
       <c r="Q53" s="1"/>
       <c r="R53" s="1"/>
     </row>
-    <row r="54" spans="1:18" ht="27.95" hidden="1" customHeight="1">
+    <row r="54" spans="1:18" ht="27.9" hidden="1" customHeight="1">
       <c r="A54" s="15">
         <v>1</v>
       </c>
@@ -4569,7 +4569,7 @@
       <c r="Q54" s="1"/>
       <c r="R54" s="1"/>
     </row>
-    <row r="55" spans="1:18" ht="27.95" hidden="1" customHeight="1">
+    <row r="55" spans="1:18" ht="27.9" hidden="1" customHeight="1">
       <c r="A55" s="15">
         <v>2</v>
       </c>
@@ -4611,7 +4611,7 @@
       <c r="Q55" s="1"/>
       <c r="R55" s="1"/>
     </row>
-    <row r="56" spans="1:18" ht="27.95" hidden="1" customHeight="1">
+    <row r="56" spans="1:18" ht="27.9" hidden="1" customHeight="1">
       <c r="A56" s="15">
         <v>3</v>
       </c>
@@ -4653,7 +4653,7 @@
       <c r="Q56" s="1"/>
       <c r="R56" s="1"/>
     </row>
-    <row r="57" spans="1:18" ht="27.95" hidden="1" customHeight="1">
+    <row r="57" spans="1:18" ht="27.9" hidden="1" customHeight="1">
       <c r="A57" s="15">
         <v>4</v>
       </c>
@@ -4695,7 +4695,7 @@
       <c r="Q57" s="1"/>
       <c r="R57" s="1"/>
     </row>
-    <row r="58" spans="1:18" ht="27.95" hidden="1" customHeight="1">
+    <row r="58" spans="1:18" ht="27.9" hidden="1" customHeight="1">
       <c r="A58" s="15">
         <v>5</v>
       </c>
@@ -4737,7 +4737,7 @@
       <c r="Q58" s="1"/>
       <c r="R58" s="1"/>
     </row>
-    <row r="59" spans="1:18" ht="27.95" hidden="1" customHeight="1">
+    <row r="59" spans="1:18" ht="27.9" hidden="1" customHeight="1">
       <c r="A59" s="15">
         <v>6</v>
       </c>
@@ -4779,7 +4779,7 @@
       <c r="Q59" s="1"/>
       <c r="R59" s="1"/>
     </row>
-    <row r="60" spans="1:18" ht="27.95" hidden="1" customHeight="1">
+    <row r="60" spans="1:18" ht="27.9" hidden="1" customHeight="1">
       <c r="A60" s="15">
         <v>7</v>
       </c>
@@ -4821,7 +4821,7 @@
       <c r="Q60" s="1"/>
       <c r="R60" s="1"/>
     </row>
-    <row r="61" spans="1:18" ht="27.95" hidden="1" customHeight="1">
+    <row r="61" spans="1:18" ht="27.9" hidden="1" customHeight="1">
       <c r="A61" s="15">
         <v>8</v>
       </c>
@@ -4863,7 +4863,7 @@
       <c r="Q61" s="1"/>
       <c r="R61" s="1"/>
     </row>
-    <row r="62" spans="1:18" ht="27.95" hidden="1" customHeight="1">
+    <row r="62" spans="1:18" ht="27.9" hidden="1" customHeight="1">
       <c r="A62" s="15">
         <v>9</v>
       </c>
@@ -4905,7 +4905,7 @@
       <c r="Q62" s="1"/>
       <c r="R62" s="1"/>
     </row>
-    <row r="63" spans="1:18" ht="27.95" hidden="1" customHeight="1">
+    <row r="63" spans="1:18" ht="27.9" hidden="1" customHeight="1">
       <c r="A63" s="15">
         <v>10</v>
       </c>
@@ -4947,7 +4947,7 @@
       <c r="Q63" s="1"/>
       <c r="R63" s="1"/>
     </row>
-    <row r="64" spans="1:18" ht="27.95" customHeight="1">
+    <row r="64" spans="1:18" ht="27.9" customHeight="1">
       <c r="A64" s="15">
         <v>11</v>
       </c>
@@ -4989,7 +4989,7 @@
       <c r="Q64" s="1"/>
       <c r="R64" s="1"/>
     </row>
-    <row r="65" spans="1:18" ht="27.95" customHeight="1">
+    <row r="65" spans="1:18" ht="27.9" customHeight="1">
       <c r="A65" s="15">
         <v>12</v>
       </c>
@@ -5031,7 +5031,7 @@
       <c r="Q65" s="1"/>
       <c r="R65" s="1"/>
     </row>
-    <row r="66" spans="1:18" ht="27.95" customHeight="1">
+    <row r="66" spans="1:18" ht="27.9" customHeight="1">
       <c r="A66" s="15">
         <v>13</v>
       </c>
@@ -5073,7 +5073,7 @@
       <c r="Q66" s="1"/>
       <c r="R66" s="1"/>
     </row>
-    <row r="67" spans="1:18" ht="27.95" customHeight="1">
+    <row r="67" spans="1:18" ht="27.9" customHeight="1">
       <c r="A67" s="15">
         <v>14</v>
       </c>
@@ -5115,7 +5115,7 @@
       <c r="Q67" s="1"/>
       <c r="R67" s="1"/>
     </row>
-    <row r="68" spans="1:18" ht="27.95" customHeight="1">
+    <row r="68" spans="1:18" ht="27.9" customHeight="1">
       <c r="A68" s="15">
         <v>15</v>
       </c>
@@ -5157,7 +5157,7 @@
       <c r="Q68" s="1"/>
       <c r="R68" s="1"/>
     </row>
-    <row r="69" spans="1:18" ht="27.95" customHeight="1">
+    <row r="69" spans="1:18" ht="27.9" customHeight="1">
       <c r="A69" s="15">
         <v>16</v>
       </c>
@@ -5199,7 +5199,7 @@
       <c r="Q69" s="1"/>
       <c r="R69" s="1"/>
     </row>
-    <row r="70" spans="1:18" ht="27.95" customHeight="1">
+    <row r="70" spans="1:18" ht="27.9" customHeight="1">
       <c r="A70" s="15">
         <v>17</v>
       </c>
@@ -5241,7 +5241,7 @@
       <c r="Q70" s="1"/>
       <c r="R70" s="1"/>
     </row>
-    <row r="71" spans="1:18" ht="27.95" customHeight="1">
+    <row r="71" spans="1:18" ht="27.9" customHeight="1">
       <c r="A71" s="15">
         <v>18</v>
       </c>
@@ -5283,7 +5283,7 @@
       <c r="Q71" s="1"/>
       <c r="R71" s="1"/>
     </row>
-    <row r="72" spans="1:18" ht="27.95" customHeight="1">
+    <row r="72" spans="1:18" ht="27.9" customHeight="1">
       <c r="A72" s="15">
         <v>19</v>
       </c>
@@ -5325,7 +5325,7 @@
       <c r="Q72" s="1"/>
       <c r="R72" s="1"/>
     </row>
-    <row r="73" spans="1:18" ht="27.95" customHeight="1">
+    <row r="73" spans="1:18" ht="27.9" customHeight="1">
       <c r="A73" s="15">
         <v>20</v>
       </c>
@@ -5367,7 +5367,7 @@
       <c r="Q73" s="1"/>
       <c r="R73" s="1"/>
     </row>
-    <row r="74" spans="1:18" ht="27.95" customHeight="1">
+    <row r="74" spans="1:18" ht="27.9" customHeight="1">
       <c r="A74" s="15">
         <v>21</v>
       </c>
@@ -5409,7 +5409,7 @@
       <c r="Q74" s="1"/>
       <c r="R74" s="1"/>
     </row>
-    <row r="75" spans="1:18" ht="27.95" customHeight="1">
+    <row r="75" spans="1:18" ht="27.9" customHeight="1">
       <c r="A75" s="20">
         <v>22</v>
       </c>
@@ -5451,7 +5451,7 @@
       <c r="Q75" s="1"/>
       <c r="R75" s="1"/>
     </row>
-    <row r="76" spans="1:18" ht="27.95" customHeight="1">
+    <row r="76" spans="1:18" ht="27.9" customHeight="1">
       <c r="A76" s="20">
         <v>23</v>
       </c>
@@ -5493,7 +5493,7 @@
       <c r="Q76" s="1"/>
       <c r="R76" s="1"/>
     </row>
-    <row r="77" spans="1:18" ht="27.95" customHeight="1">
+    <row r="77" spans="1:18" ht="27.9" customHeight="1">
       <c r="A77" s="15"/>
       <c r="B77" s="7"/>
       <c r="C77" s="7"/>
@@ -5513,7 +5513,7 @@
       <c r="Q77" s="1"/>
       <c r="R77" s="1"/>
     </row>
-    <row r="78" spans="1:18" ht="27.95" customHeight="1">
+    <row r="78" spans="1:18" ht="27.9" customHeight="1">
       <c r="A78" s="15"/>
       <c r="B78" s="7"/>
       <c r="C78" s="7"/>
@@ -5533,7 +5533,7 @@
       <c r="Q78" s="1"/>
       <c r="R78" s="1"/>
     </row>
-    <row r="79" spans="1:18" ht="27.95" customHeight="1">
+    <row r="79" spans="1:18" ht="27.9" customHeight="1">
       <c r="A79" s="15"/>
       <c r="B79" s="7"/>
       <c r="C79" s="7"/>
@@ -5553,7 +5553,7 @@
       <c r="Q79" s="1"/>
       <c r="R79" s="1"/>
     </row>
-    <row r="80" spans="1:18" ht="27.95" customHeight="1">
+    <row r="80" spans="1:18" ht="27.9" customHeight="1">
       <c r="A80" s="15"/>
       <c r="B80" s="7"/>
       <c r="C80" s="7"/>
@@ -5573,7 +5573,7 @@
       <c r="Q80" s="1"/>
       <c r="R80" s="1"/>
     </row>
-    <row r="81" spans="1:18" ht="27.95" customHeight="1">
+    <row r="81" spans="1:18" ht="27.9" customHeight="1">
       <c r="A81" s="15"/>
       <c r="B81" s="7"/>
       <c r="C81" s="7"/>
@@ -5593,7 +5593,7 @@
       <c r="Q81" s="1"/>
       <c r="R81" s="1"/>
     </row>
-    <row r="82" spans="1:18" ht="27.95" customHeight="1">
+    <row r="82" spans="1:18" ht="27.9" customHeight="1">
       <c r="A82" s="15"/>
       <c r="B82" s="7"/>
       <c r="C82" s="7"/>
@@ -5613,7 +5613,7 @@
       <c r="Q82" s="1"/>
       <c r="R82" s="1"/>
     </row>
-    <row r="83" spans="1:18" ht="27.95" customHeight="1">
+    <row r="83" spans="1:18" ht="27.9" customHeight="1">
       <c r="A83" s="15"/>
       <c r="B83" s="7"/>
       <c r="C83" s="7"/>
@@ -5633,7 +5633,7 @@
       <c r="Q83" s="1"/>
       <c r="R83" s="1"/>
     </row>
-    <row r="84" spans="1:18" ht="27.95" customHeight="1">
+    <row r="84" spans="1:18" ht="27.9" customHeight="1">
       <c r="A84" s="15"/>
       <c r="B84" s="7"/>
       <c r="C84" s="7"/>
@@ -5653,7 +5653,7 @@
       <c r="Q84" s="1"/>
       <c r="R84" s="1"/>
     </row>
-    <row r="85" spans="1:18" ht="27.95" customHeight="1">
+    <row r="85" spans="1:18" ht="27.9" customHeight="1">
       <c r="A85" s="15"/>
       <c r="B85" s="7"/>
       <c r="C85" s="7"/>
@@ -5673,7 +5673,7 @@
       <c r="Q85" s="1"/>
       <c r="R85" s="1"/>
     </row>
-    <row r="86" spans="1:18" ht="27.95" customHeight="1">
+    <row r="86" spans="1:18" ht="27.9" customHeight="1">
       <c r="A86" s="15"/>
       <c r="B86" s="7"/>
       <c r="C86" s="7"/>
@@ -5693,7 +5693,7 @@
       <c r="Q86" s="1"/>
       <c r="R86" s="1"/>
     </row>
-    <row r="87" spans="1:18" ht="27.95" customHeight="1">
+    <row r="87" spans="1:18" ht="27.9" customHeight="1">
       <c r="A87" s="15"/>
       <c r="B87" s="7"/>
       <c r="C87" s="7"/>
@@ -5713,7 +5713,7 @@
       <c r="Q87" s="1"/>
       <c r="R87" s="1"/>
     </row>
-    <row r="88" spans="1:18" ht="27.95" customHeight="1">
+    <row r="88" spans="1:18" ht="27.9" customHeight="1">
       <c r="A88" s="15"/>
       <c r="B88" s="7"/>
       <c r="C88" s="7"/>
@@ -5733,7 +5733,7 @@
       <c r="Q88" s="1"/>
       <c r="R88" s="1"/>
     </row>
-    <row r="89" spans="1:18" ht="27.95" customHeight="1">
+    <row r="89" spans="1:18" ht="27.9" customHeight="1">
       <c r="A89" s="15"/>
       <c r="B89" s="7"/>
       <c r="C89" s="7"/>
@@ -5753,7 +5753,7 @@
       <c r="Q89" s="1"/>
       <c r="R89" s="1"/>
     </row>
-    <row r="90" spans="1:18" ht="27.95" customHeight="1">
+    <row r="90" spans="1:18" ht="27.9" customHeight="1">
       <c r="A90" s="15"/>
       <c r="B90" s="7"/>
       <c r="C90" s="7"/>
@@ -5773,7 +5773,7 @@
       <c r="Q90" s="1"/>
       <c r="R90" s="1"/>
     </row>
-    <row r="91" spans="1:18" ht="27.95" customHeight="1">
+    <row r="91" spans="1:18" ht="27.9" customHeight="1">
       <c r="A91" s="15"/>
       <c r="B91" s="7"/>
       <c r="C91" s="7"/>
@@ -5793,7 +5793,7 @@
       <c r="Q91" s="1"/>
       <c r="R91" s="1"/>
     </row>
-    <row r="92" spans="1:18" ht="27.95" customHeight="1">
+    <row r="92" spans="1:18" ht="27.9" customHeight="1">
       <c r="A92" s="15"/>
       <c r="B92" s="7"/>
       <c r="C92" s="7"/>
@@ -5813,7 +5813,7 @@
       <c r="Q92" s="1"/>
       <c r="R92" s="1"/>
     </row>
-    <row r="93" spans="1:18" ht="27.95" customHeight="1">
+    <row r="93" spans="1:18" ht="27.9" customHeight="1">
       <c r="A93" s="15"/>
       <c r="B93" s="7"/>
       <c r="C93" s="7"/>
@@ -5833,7 +5833,7 @@
       <c r="Q93" s="1"/>
       <c r="R93" s="1"/>
     </row>
-    <row r="94" spans="1:18" ht="27.95" customHeight="1">
+    <row r="94" spans="1:18" ht="27.9" customHeight="1">
       <c r="A94" s="15"/>
       <c r="B94" s="7"/>
       <c r="C94" s="7"/>
@@ -5853,7 +5853,7 @@
       <c r="Q94" s="1"/>
       <c r="R94" s="1"/>
     </row>
-    <row r="95" spans="1:18" ht="27.95" customHeight="1">
+    <row r="95" spans="1:18" ht="27.9" customHeight="1">
       <c r="A95" s="15"/>
       <c r="B95" s="7"/>
       <c r="C95" s="7"/>
@@ -5873,7 +5873,7 @@
       <c r="Q95" s="1"/>
       <c r="R95" s="1"/>
     </row>
-    <row r="96" spans="1:18" ht="27.95" customHeight="1">
+    <row r="96" spans="1:18" ht="27.9" customHeight="1">
       <c r="A96" s="15"/>
       <c r="B96" s="7"/>
       <c r="C96" s="7"/>
@@ -5893,7 +5893,7 @@
       <c r="Q96" s="1"/>
       <c r="R96" s="1"/>
     </row>
-    <row r="97" spans="1:18" ht="27.95" customHeight="1">
+    <row r="97" spans="1:18" ht="27.9" customHeight="1">
       <c r="A97" s="15"/>
       <c r="B97" s="7"/>
       <c r="C97" s="7"/>
@@ -5913,7 +5913,7 @@
       <c r="Q97" s="1"/>
       <c r="R97" s="1"/>
     </row>
-    <row r="98" spans="1:18" ht="27.95" customHeight="1">
+    <row r="98" spans="1:18" ht="27.9" customHeight="1">
       <c r="A98" s="15"/>
       <c r="B98" s="7"/>
       <c r="C98" s="7"/>
@@ -5933,7 +5933,7 @@
       <c r="Q98" s="1"/>
       <c r="R98" s="1"/>
     </row>
-    <row r="99" spans="1:18" ht="27.95" customHeight="1">
+    <row r="99" spans="1:18" ht="27.9" customHeight="1">
       <c r="A99" s="15"/>
       <c r="B99" s="7"/>
       <c r="C99" s="7"/>
@@ -5953,7 +5953,7 @@
       <c r="Q99" s="1"/>
       <c r="R99" s="1"/>
     </row>
-    <row r="100" spans="1:18" ht="27.95" customHeight="1">
+    <row r="100" spans="1:18" ht="27.9" customHeight="1">
       <c r="A100" s="15"/>
       <c r="B100" s="7"/>
       <c r="C100" s="7"/>
@@ -5973,7 +5973,7 @@
       <c r="Q100" s="1"/>
       <c r="R100" s="1"/>
     </row>
-    <row r="101" spans="1:18" ht="27.95" customHeight="1">
+    <row r="101" spans="1:18" ht="27.9" customHeight="1">
       <c r="A101" s="15"/>
       <c r="B101" s="7"/>
       <c r="C101" s="7"/>
@@ -5993,7 +5993,7 @@
       <c r="Q101" s="1"/>
       <c r="R101" s="1"/>
     </row>
-    <row r="102" spans="1:18" ht="27.95" customHeight="1">
+    <row r="102" spans="1:18" ht="27.9" customHeight="1">
       <c r="A102" s="15"/>
       <c r="B102" s="7"/>
       <c r="C102" s="7"/>
@@ -6013,7 +6013,7 @@
       <c r="Q102" s="1"/>
       <c r="R102" s="1"/>
     </row>
-    <row r="103" spans="1:18" ht="27.95" customHeight="1">
+    <row r="103" spans="1:18" ht="27.9" customHeight="1">
       <c r="A103" s="15"/>
       <c r="B103" s="7"/>
       <c r="C103" s="7"/>
@@ -6033,7 +6033,7 @@
       <c r="Q103" s="1"/>
       <c r="R103" s="1"/>
     </row>
-    <row r="104" spans="1:18" ht="27.95" customHeight="1">
+    <row r="104" spans="1:18" ht="27.9" customHeight="1">
       <c r="A104" s="15"/>
       <c r="B104" s="7"/>
       <c r="C104" s="7"/>
@@ -6053,7 +6053,7 @@
       <c r="Q104" s="1"/>
       <c r="R104" s="1"/>
     </row>
-    <row r="105" spans="1:18" ht="27.95" customHeight="1">
+    <row r="105" spans="1:18" ht="27.9" customHeight="1">
       <c r="A105" s="15"/>
       <c r="B105" s="7"/>
       <c r="C105" s="7"/>
@@ -6073,7 +6073,7 @@
       <c r="Q105" s="1"/>
       <c r="R105" s="1"/>
     </row>
-    <row r="106" spans="1:18" ht="27.95" customHeight="1">
+    <row r="106" spans="1:18" ht="27.9" customHeight="1">
       <c r="A106" s="15"/>
       <c r="B106" s="7"/>
       <c r="C106" s="7"/>
@@ -6093,7 +6093,7 @@
       <c r="Q106" s="1"/>
       <c r="R106" s="1"/>
     </row>
-    <row r="107" spans="1:18" ht="27.95" customHeight="1">
+    <row r="107" spans="1:18" ht="27.9" customHeight="1">
       <c r="A107" s="15"/>
       <c r="B107" s="7"/>
       <c r="C107" s="7"/>
@@ -6113,7 +6113,7 @@
       <c r="Q107" s="1"/>
       <c r="R107" s="1"/>
     </row>
-    <row r="108" spans="1:18" ht="27.95" customHeight="1">
+    <row r="108" spans="1:18" ht="27.9" customHeight="1">
       <c r="A108" s="15"/>
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
@@ -6133,7 +6133,7 @@
       <c r="Q108" s="1"/>
       <c r="R108" s="1"/>
     </row>
-    <row r="109" spans="1:18" ht="27.95" customHeight="1">
+    <row r="109" spans="1:18" ht="27.9" customHeight="1">
       <c r="A109" s="15"/>
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
@@ -6153,7 +6153,7 @@
       <c r="Q109" s="1"/>
       <c r="R109" s="1"/>
     </row>
-    <row r="110" spans="1:18" ht="27.95" customHeight="1">
+    <row r="110" spans="1:18" ht="27.9" customHeight="1">
       <c r="A110" s="15"/>
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
@@ -6173,7 +6173,7 @@
       <c r="Q110" s="1"/>
       <c r="R110" s="1"/>
     </row>
-    <row r="111" spans="1:18" ht="27.95" customHeight="1">
+    <row r="111" spans="1:18" ht="27.9" customHeight="1">
       <c r="A111" s="15"/>
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
@@ -6193,7 +6193,7 @@
       <c r="Q111" s="1"/>
       <c r="R111" s="1"/>
     </row>
-    <row r="112" spans="1:18" ht="27.95" customHeight="1">
+    <row r="112" spans="1:18" ht="27.9" customHeight="1">
       <c r="A112" s="15"/>
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
@@ -6213,7 +6213,7 @@
       <c r="Q112" s="1"/>
       <c r="R112" s="1"/>
     </row>
-    <row r="113" spans="1:18" ht="27.95" customHeight="1">
+    <row r="113" spans="1:18" ht="27.9" customHeight="1">
       <c r="A113" s="15"/>
       <c r="B113" s="7"/>
       <c r="C113" s="7"/>
@@ -6233,7 +6233,7 @@
       <c r="Q113" s="1"/>
       <c r="R113" s="1"/>
     </row>
-    <row r="114" spans="1:18" ht="27.95" customHeight="1">
+    <row r="114" spans="1:18" ht="27.9" customHeight="1">
       <c r="A114" s="15"/>
       <c r="B114" s="7"/>
       <c r="C114" s="7"/>
@@ -6253,7 +6253,7 @@
       <c r="Q114" s="1"/>
       <c r="R114" s="1"/>
     </row>
-    <row r="115" spans="1:18" ht="27.95" customHeight="1">
+    <row r="115" spans="1:18" ht="27.9" customHeight="1">
       <c r="A115" s="15"/>
       <c r="B115" s="7"/>
       <c r="C115" s="7"/>
@@ -6273,7 +6273,7 @@
       <c r="Q115" s="1"/>
       <c r="R115" s="1"/>
     </row>
-    <row r="116" spans="1:18" ht="27.95" customHeight="1">
+    <row r="116" spans="1:18" ht="27.9" customHeight="1">
       <c r="A116" s="15"/>
       <c r="B116" s="7"/>
       <c r="C116" s="7"/>
@@ -6293,7 +6293,7 @@
       <c r="Q116" s="1"/>
       <c r="R116" s="1"/>
     </row>
-    <row r="117" spans="1:18" ht="27.95" customHeight="1">
+    <row r="117" spans="1:18" ht="27.9" customHeight="1">
       <c r="A117" s="15"/>
       <c r="B117" s="7"/>
       <c r="C117" s="7"/>
@@ -6313,7 +6313,7 @@
       <c r="Q117" s="1"/>
       <c r="R117" s="1"/>
     </row>
-    <row r="118" spans="1:18" ht="27.95" customHeight="1">
+    <row r="118" spans="1:18" ht="27.9" customHeight="1">
       <c r="A118" s="15"/>
       <c r="B118" s="7"/>
       <c r="C118" s="7"/>
@@ -6333,7 +6333,7 @@
       <c r="Q118" s="1"/>
       <c r="R118" s="1"/>
     </row>
-    <row r="119" spans="1:18" ht="27.95" customHeight="1">
+    <row r="119" spans="1:18" ht="27.9" customHeight="1">
       <c r="A119" s="15"/>
       <c r="B119" s="7"/>
       <c r="C119" s="7"/>
@@ -6353,7 +6353,7 @@
       <c r="Q119" s="1"/>
       <c r="R119" s="1"/>
     </row>
-    <row r="120" spans="1:18" ht="27.95" customHeight="1">
+    <row r="120" spans="1:18" ht="27.9" customHeight="1">
       <c r="A120" s="15"/>
       <c r="B120" s="7"/>
       <c r="C120" s="7"/>
@@ -6373,7 +6373,7 @@
       <c r="Q120" s="1"/>
       <c r="R120" s="1"/>
     </row>
-    <row r="121" spans="1:18" ht="27.95" customHeight="1">
+    <row r="121" spans="1:18" ht="27.9" customHeight="1">
       <c r="A121" s="15"/>
       <c r="B121" s="7"/>
       <c r="C121" s="7"/>
@@ -6393,7 +6393,7 @@
       <c r="Q121" s="1"/>
       <c r="R121" s="1"/>
     </row>
-    <row r="122" spans="1:18" ht="27.95" customHeight="1">
+    <row r="122" spans="1:18" ht="27.9" customHeight="1">
       <c r="A122" s="15"/>
       <c r="B122" s="7"/>
       <c r="C122" s="7"/>
@@ -6413,7 +6413,7 @@
       <c r="Q122" s="1"/>
       <c r="R122" s="1"/>
     </row>
-    <row r="123" spans="1:18" ht="27.95" customHeight="1">
+    <row r="123" spans="1:18" ht="27.9" customHeight="1">
       <c r="A123" s="15"/>
       <c r="B123" s="7"/>
       <c r="C123" s="7"/>
@@ -6433,7 +6433,7 @@
       <c r="Q123" s="1"/>
       <c r="R123" s="1"/>
     </row>
-    <row r="124" spans="1:18" ht="27.95" customHeight="1">
+    <row r="124" spans="1:18" ht="27.9" customHeight="1">
       <c r="A124" s="15"/>
       <c r="B124" s="7"/>
       <c r="C124" s="7"/>
@@ -6453,7 +6453,7 @@
       <c r="Q124" s="1"/>
       <c r="R124" s="1"/>
     </row>
-    <row r="125" spans="1:18" ht="27.95" customHeight="1">
+    <row r="125" spans="1:18" ht="27.9" customHeight="1">
       <c r="A125" s="15"/>
       <c r="B125" s="7"/>
       <c r="C125" s="7"/>
@@ -6473,7 +6473,7 @@
       <c r="Q125" s="1"/>
       <c r="R125" s="1"/>
     </row>
-    <row r="126" spans="1:18" ht="27.95" customHeight="1">
+    <row r="126" spans="1:18" ht="27.9" customHeight="1">
       <c r="A126" s="15"/>
       <c r="B126" s="7"/>
       <c r="C126" s="7"/>
@@ -6493,7 +6493,7 @@
       <c r="Q126" s="1"/>
       <c r="R126" s="1"/>
     </row>
-    <row r="127" spans="1:18" ht="27.95" customHeight="1">
+    <row r="127" spans="1:18" ht="27.9" customHeight="1">
       <c r="A127" s="15"/>
       <c r="B127" s="7"/>
       <c r="C127" s="7"/>
@@ -6513,7 +6513,7 @@
       <c r="Q127" s="1"/>
       <c r="R127" s="1"/>
     </row>
-    <row r="128" spans="1:18" ht="27.95" customHeight="1">
+    <row r="128" spans="1:18" ht="27.9" customHeight="1">
       <c r="A128" s="15"/>
       <c r="B128" s="7"/>
       <c r="C128" s="7"/>
@@ -6533,7 +6533,7 @@
       <c r="Q128" s="1"/>
       <c r="R128" s="1"/>
     </row>
-    <row r="129" spans="1:18" ht="27.95" customHeight="1">
+    <row r="129" spans="1:18" ht="27.9" customHeight="1">
       <c r="A129" s="15"/>
       <c r="B129" s="7"/>
       <c r="C129" s="7"/>
@@ -6553,7 +6553,7 @@
       <c r="Q129" s="1"/>
       <c r="R129" s="1"/>
     </row>
-    <row r="130" spans="1:18" ht="27.95" customHeight="1">
+    <row r="130" spans="1:18" ht="27.9" customHeight="1">
       <c r="A130" s="15"/>
       <c r="B130" s="7"/>
       <c r="C130" s="7"/>
@@ -6573,7 +6573,7 @@
       <c r="Q130" s="1"/>
       <c r="R130" s="1"/>
     </row>
-    <row r="131" spans="1:18" ht="27.95" customHeight="1">
+    <row r="131" spans="1:18" ht="27.9" customHeight="1">
       <c r="A131" s="15"/>
       <c r="B131" s="7"/>
       <c r="C131" s="7"/>
@@ -6593,7 +6593,7 @@
       <c r="Q131" s="1"/>
       <c r="R131" s="1"/>
     </row>
-    <row r="132" spans="1:18" ht="27.95" customHeight="1">
+    <row r="132" spans="1:18" ht="27.9" customHeight="1">
       <c r="A132" s="15"/>
       <c r="B132" s="7"/>
       <c r="C132" s="7"/>
@@ -6613,7 +6613,7 @@
       <c r="Q132" s="1"/>
       <c r="R132" s="1"/>
     </row>
-    <row r="133" spans="1:18" ht="27.95" customHeight="1">
+    <row r="133" spans="1:18" ht="27.9" customHeight="1">
       <c r="A133" s="15"/>
       <c r="B133" s="7"/>
       <c r="C133" s="7"/>
@@ -6633,7 +6633,7 @@
       <c r="Q133" s="1"/>
       <c r="R133" s="1"/>
     </row>
-    <row r="134" spans="1:18" ht="27.95" customHeight="1">
+    <row r="134" spans="1:18" ht="27.9" customHeight="1">
       <c r="A134" s="15"/>
       <c r="B134" s="7"/>
       <c r="C134" s="7"/>
@@ -6653,7 +6653,7 @@
       <c r="Q134" s="1"/>
       <c r="R134" s="1"/>
     </row>
-    <row r="135" spans="1:18" ht="27.95" customHeight="1">
+    <row r="135" spans="1:18" ht="27.9" customHeight="1">
       <c r="A135" s="15"/>
       <c r="B135" s="7"/>
       <c r="C135" s="7"/>
@@ -6673,7 +6673,7 @@
       <c r="Q135" s="1"/>
       <c r="R135" s="1"/>
     </row>
-    <row r="136" spans="1:18" ht="27.95" customHeight="1">
+    <row r="136" spans="1:18" ht="27.9" customHeight="1">
       <c r="A136" s="15"/>
       <c r="B136" s="7"/>
       <c r="C136" s="7"/>
@@ -6693,7 +6693,7 @@
       <c r="Q136" s="1"/>
       <c r="R136" s="1"/>
     </row>
-    <row r="137" spans="1:18" ht="27.95" customHeight="1">
+    <row r="137" spans="1:18" ht="27.9" customHeight="1">
       <c r="A137" s="15"/>
       <c r="B137" s="7"/>
       <c r="C137" s="7"/>
@@ -6713,7 +6713,7 @@
       <c r="Q137" s="1"/>
       <c r="R137" s="1"/>
     </row>
-    <row r="138" spans="1:18" ht="27.95" customHeight="1">
+    <row r="138" spans="1:18" ht="27.9" customHeight="1">
       <c r="A138" s="15"/>
       <c r="B138" s="7"/>
       <c r="C138" s="7"/>
@@ -6733,7 +6733,7 @@
       <c r="Q138" s="1"/>
       <c r="R138" s="1"/>
     </row>
-    <row r="139" spans="1:18" ht="27.95" customHeight="1">
+    <row r="139" spans="1:18" ht="27.9" customHeight="1">
       <c r="A139" s="15"/>
       <c r="B139" s="7"/>
       <c r="C139" s="7"/>
@@ -6753,7 +6753,7 @@
       <c r="Q139" s="1"/>
       <c r="R139" s="1"/>
     </row>
-    <row r="140" spans="1:18" ht="27.95" customHeight="1">
+    <row r="140" spans="1:18" ht="27.9" customHeight="1">
       <c r="A140" s="15"/>
       <c r="B140" s="7"/>
       <c r="C140" s="7"/>
@@ -6773,7 +6773,7 @@
       <c r="Q140" s="1"/>
       <c r="R140" s="1"/>
     </row>
-    <row r="141" spans="1:18" ht="27.95" customHeight="1">
+    <row r="141" spans="1:18" ht="27.9" customHeight="1">
       <c r="A141" s="15"/>
       <c r="B141" s="7"/>
       <c r="C141" s="7"/>
@@ -6793,7 +6793,7 @@
       <c r="Q141" s="1"/>
       <c r="R141" s="1"/>
     </row>
-    <row r="142" spans="1:18" ht="27.95" customHeight="1">
+    <row r="142" spans="1:18" ht="27.9" customHeight="1">
       <c r="A142" s="15"/>
       <c r="B142" s="7"/>
       <c r="C142" s="7"/>
@@ -6813,7 +6813,7 @@
       <c r="Q142" s="1"/>
       <c r="R142" s="1"/>
     </row>
-    <row r="143" spans="1:18" ht="27.95" customHeight="1">
+    <row r="143" spans="1:18" ht="27.9" customHeight="1">
       <c r="A143" s="15"/>
       <c r="B143" s="7"/>
       <c r="C143" s="7"/>
@@ -6833,7 +6833,7 @@
       <c r="Q143" s="1"/>
       <c r="R143" s="1"/>
     </row>
-    <row r="144" spans="1:18" ht="27.95" customHeight="1">
+    <row r="144" spans="1:18" ht="27.9" customHeight="1">
       <c r="A144" s="15"/>
       <c r="B144" s="7"/>
       <c r="C144" s="7"/>
@@ -6853,7 +6853,7 @@
       <c r="Q144" s="1"/>
       <c r="R144" s="1"/>
     </row>
-    <row r="145" spans="1:18" ht="27.95" customHeight="1">
+    <row r="145" spans="1:18" ht="27.9" customHeight="1">
       <c r="A145" s="15"/>
       <c r="B145" s="7"/>
       <c r="C145" s="7"/>
@@ -6873,7 +6873,7 @@
       <c r="Q145" s="1"/>
       <c r="R145" s="1"/>
     </row>
-    <row r="146" spans="1:18" ht="27.95" customHeight="1">
+    <row r="146" spans="1:18" ht="27.9" customHeight="1">
       <c r="A146" s="15"/>
       <c r="B146" s="7"/>
       <c r="C146" s="7"/>
@@ -6893,7 +6893,7 @@
       <c r="Q146" s="1"/>
       <c r="R146" s="1"/>
     </row>
-    <row r="147" spans="1:18" ht="27.95" customHeight="1">
+    <row r="147" spans="1:18" ht="27.9" customHeight="1">
       <c r="A147" s="15"/>
       <c r="B147" s="7"/>
       <c r="C147" s="7"/>
@@ -6913,7 +6913,7 @@
       <c r="Q147" s="1"/>
       <c r="R147" s="1"/>
     </row>
-    <row r="148" spans="1:18" ht="27.95" customHeight="1">
+    <row r="148" spans="1:18" ht="27.9" customHeight="1">
       <c r="A148" s="15"/>
       <c r="B148" s="7"/>
       <c r="C148" s="7"/>
@@ -6933,7 +6933,7 @@
       <c r="Q148" s="1"/>
       <c r="R148" s="1"/>
     </row>
-    <row r="149" spans="1:18" ht="27.95" customHeight="1">
+    <row r="149" spans="1:18" ht="27.9" customHeight="1">
       <c r="A149" s="15"/>
       <c r="B149" s="7"/>
       <c r="C149" s="7"/>
@@ -6953,7 +6953,7 @@
       <c r="Q149" s="1"/>
       <c r="R149" s="1"/>
     </row>
-    <row r="150" spans="1:18" ht="27.95" customHeight="1">
+    <row r="150" spans="1:18" ht="27.9" customHeight="1">
       <c r="A150" s="15"/>
       <c r="B150" s="7"/>
       <c r="C150" s="7"/>
@@ -6973,7 +6973,7 @@
       <c r="Q150" s="1"/>
       <c r="R150" s="1"/>
     </row>
-    <row r="151" spans="1:18" ht="27.95" customHeight="1">
+    <row r="151" spans="1:18" ht="27.9" customHeight="1">
       <c r="A151" s="15"/>
       <c r="B151" s="7"/>
       <c r="C151" s="7"/>
@@ -6993,7 +6993,7 @@
       <c r="Q151" s="1"/>
       <c r="R151" s="1"/>
     </row>
-    <row r="152" spans="1:18" ht="27.95" customHeight="1">
+    <row r="152" spans="1:18" ht="27.9" customHeight="1">
       <c r="A152" s="15"/>
       <c r="B152" s="7"/>
       <c r="C152" s="7"/>
@@ -7013,7 +7013,7 @@
       <c r="Q152" s="1"/>
       <c r="R152" s="1"/>
     </row>
-    <row r="153" spans="1:18" ht="27.95" customHeight="1">
+    <row r="153" spans="1:18" ht="27.9" customHeight="1">
       <c r="A153" s="15"/>
       <c r="B153" s="7"/>
       <c r="C153" s="7"/>
@@ -7073,7 +7073,7 @@
       <c r="Q155" s="1"/>
       <c r="R155" s="1"/>
     </row>
-    <row r="156" spans="1:18" ht="21.95" customHeight="1">
+    <row r="156" spans="1:18" ht="21.9" customHeight="1">
       <c r="A156" s="15"/>
       <c r="B156" s="7"/>
       <c r="C156" s="7"/>
@@ -7092,7 +7092,7 @@
       <c r="P156" s="1"/>
       <c r="Q156" s="1"/>
     </row>
-    <row r="157" spans="1:18" ht="33.950000000000003" customHeight="1">
+    <row r="157" spans="1:18" ht="33.9" customHeight="1">
       <c r="A157" s="15"/>
       <c r="B157" s="7"/>
       <c r="C157" s="7"/>
@@ -7111,7 +7111,7 @@
       <c r="P157" s="1"/>
       <c r="Q157" s="1"/>
     </row>
-    <row r="158" spans="1:18" ht="39.950000000000003" customHeight="1">
+    <row r="158" spans="1:18" ht="39.9" customHeight="1">
       <c r="A158" s="15"/>
       <c r="B158" s="7"/>
       <c r="C158" s="7"/>
@@ -7244,16 +7244,16 @@
       <c r="Q164" s="1"/>
     </row>
     <row r="165" spans="1:18" ht="30" customHeight="1">
-      <c r="A165" s="40" t="s">
+      <c r="A165" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="B165" s="41"/>
-      <c r="C165" s="41"/>
-      <c r="D165" s="41"/>
-      <c r="E165" s="41"/>
-      <c r="F165" s="41"/>
-      <c r="G165" s="41"/>
-      <c r="H165" s="42"/>
+      <c r="B165" s="29"/>
+      <c r="C165" s="29"/>
+      <c r="D165" s="29"/>
+      <c r="E165" s="29"/>
+      <c r="F165" s="29"/>
+      <c r="G165" s="29"/>
+      <c r="H165" s="30"/>
       <c r="I165" s="1"/>
       <c r="J165" s="1"/>
       <c r="K165" s="1"/>
@@ -7265,16 +7265,16 @@
       <c r="Q165" s="1"/>
     </row>
     <row r="166" spans="1:18" ht="30" customHeight="1">
-      <c r="A166" s="43" t="s">
+      <c r="A166" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="B166" s="44"/>
-      <c r="C166" s="44"/>
-      <c r="D166" s="44"/>
-      <c r="E166" s="44"/>
-      <c r="F166" s="44"/>
-      <c r="G166" s="44"/>
-      <c r="H166" s="45"/>
+      <c r="B166" s="32"/>
+      <c r="C166" s="32"/>
+      <c r="D166" s="32"/>
+      <c r="E166" s="32"/>
+      <c r="F166" s="32"/>
+      <c r="G166" s="32"/>
+      <c r="H166" s="33"/>
       <c r="I166" s="1"/>
       <c r="J166" s="1"/>
       <c r="K166" s="1"/>
@@ -8301,34 +8301,54 @@
     </row>
   </sheetData>
   <mergeCells count="92">
-    <mergeCell ref="O34:R34"/>
-    <mergeCell ref="K34:N34"/>
-    <mergeCell ref="G34:J34"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C43:F43"/>
-    <mergeCell ref="G43:J43"/>
-    <mergeCell ref="K43:N43"/>
-    <mergeCell ref="O43:R43"/>
-    <mergeCell ref="A165:H165"/>
-    <mergeCell ref="A166:H166"/>
-    <mergeCell ref="C48:F48"/>
-    <mergeCell ref="G48:J48"/>
-    <mergeCell ref="K48:N48"/>
-    <mergeCell ref="O48:R48"/>
-    <mergeCell ref="A51:K51"/>
-    <mergeCell ref="A52:K52"/>
-    <mergeCell ref="C45:F45"/>
-    <mergeCell ref="G45:J45"/>
-    <mergeCell ref="K45:N45"/>
-    <mergeCell ref="O45:R45"/>
-    <mergeCell ref="C46:F46"/>
-    <mergeCell ref="G46:J46"/>
-    <mergeCell ref="K46:N46"/>
-    <mergeCell ref="O46:R46"/>
-    <mergeCell ref="K47:N47"/>
-    <mergeCell ref="G47:J47"/>
-    <mergeCell ref="C47:F47"/>
-    <mergeCell ref="O47:R47"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A27:R27"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="K28:N28"/>
+    <mergeCell ref="O28:R28"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="K29:N29"/>
+    <mergeCell ref="O29:R29"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="K30:N30"/>
+    <mergeCell ref="O30:R30"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="K33:N33"/>
+    <mergeCell ref="O33:R33"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="K31:N31"/>
+    <mergeCell ref="O31:R31"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="G35:J35"/>
+    <mergeCell ref="K35:N35"/>
+    <mergeCell ref="O35:R35"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="G36:J36"/>
+    <mergeCell ref="K36:N36"/>
+    <mergeCell ref="O36:R36"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="G37:J37"/>
+    <mergeCell ref="K37:N37"/>
+    <mergeCell ref="O37:R37"/>
+    <mergeCell ref="C38:F38"/>
+    <mergeCell ref="G38:J38"/>
+    <mergeCell ref="K38:N38"/>
+    <mergeCell ref="O38:R38"/>
+    <mergeCell ref="C39:F39"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="K39:N39"/>
+    <mergeCell ref="O39:R39"/>
+    <mergeCell ref="C40:F40"/>
+    <mergeCell ref="G40:J40"/>
+    <mergeCell ref="K40:N40"/>
+    <mergeCell ref="O40:R40"/>
     <mergeCell ref="C44:F44"/>
     <mergeCell ref="G44:J44"/>
     <mergeCell ref="K44:N44"/>
@@ -8341,58 +8361,38 @@
     <mergeCell ref="G42:J42"/>
     <mergeCell ref="K42:N42"/>
     <mergeCell ref="O42:R42"/>
-    <mergeCell ref="C39:F39"/>
-    <mergeCell ref="G39:J39"/>
-    <mergeCell ref="K39:N39"/>
-    <mergeCell ref="O39:R39"/>
-    <mergeCell ref="C40:F40"/>
-    <mergeCell ref="G40:J40"/>
-    <mergeCell ref="K40:N40"/>
-    <mergeCell ref="O40:R40"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="G37:J37"/>
-    <mergeCell ref="K37:N37"/>
-    <mergeCell ref="O37:R37"/>
-    <mergeCell ref="C38:F38"/>
-    <mergeCell ref="G38:J38"/>
-    <mergeCell ref="K38:N38"/>
-    <mergeCell ref="O38:R38"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="G35:J35"/>
-    <mergeCell ref="K35:N35"/>
-    <mergeCell ref="O35:R35"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="G36:J36"/>
-    <mergeCell ref="K36:N36"/>
-    <mergeCell ref="O36:R36"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="G33:J33"/>
-    <mergeCell ref="K33:N33"/>
-    <mergeCell ref="O33:R33"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="K31:N31"/>
-    <mergeCell ref="O31:R31"/>
+    <mergeCell ref="O48:R48"/>
+    <mergeCell ref="A51:K51"/>
+    <mergeCell ref="A52:K52"/>
+    <mergeCell ref="C45:F45"/>
+    <mergeCell ref="G45:J45"/>
+    <mergeCell ref="K45:N45"/>
+    <mergeCell ref="O45:R45"/>
+    <mergeCell ref="C46:F46"/>
+    <mergeCell ref="G46:J46"/>
+    <mergeCell ref="K46:N46"/>
+    <mergeCell ref="O46:R46"/>
+    <mergeCell ref="A165:H165"/>
+    <mergeCell ref="A166:H166"/>
+    <mergeCell ref="C48:F48"/>
+    <mergeCell ref="G48:J48"/>
+    <mergeCell ref="K48:N48"/>
+    <mergeCell ref="K47:N47"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="C47:F47"/>
+    <mergeCell ref="O47:R47"/>
     <mergeCell ref="O32:R32"/>
     <mergeCell ref="K32:N32"/>
     <mergeCell ref="G32:J32"/>
     <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="K29:N29"/>
-    <mergeCell ref="O29:R29"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="K30:N30"/>
-    <mergeCell ref="O30:R30"/>
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A27:R27"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="K28:N28"/>
-    <mergeCell ref="O28:R28"/>
+    <mergeCell ref="O34:R34"/>
+    <mergeCell ref="K34:N34"/>
+    <mergeCell ref="G34:J34"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C43:F43"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="K43:N43"/>
+    <mergeCell ref="O43:R43"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="6">
@@ -8430,7 +8430,7 @@
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
   <dimension ref="A1:D39"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="3" width="15" customWidth="1"/>
@@ -8438,30 +8438,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26.1" customHeight="1">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="C1" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="D1" s="42" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="33.950000000000003" customHeight="1">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:4" ht="33.9" customHeight="1">
+      <c r="A2" s="43" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="40" t="s">
         <v>72</v>
       </c>
     </row>
@@ -8485,7 +8485,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="5" spans="1:4" ht="33.9" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>76</v>
       </c>
@@ -8500,7 +8500,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="6" spans="1:4" ht="33.9" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>79</v>
       </c>
@@ -8515,7 +8515,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="7" spans="1:4" ht="33.9" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>81</v>
       </c>
@@ -8530,7 +8530,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="8" spans="1:4" ht="33.9" customHeight="1">
       <c r="A8" s="4" t="s">
         <v>83</v>
       </c>
@@ -8546,7 +8546,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="9" spans="1:4" ht="33.9" customHeight="1">
       <c r="A9" s="4" t="s">
         <v>85</v>
       </c>
@@ -8562,7 +8562,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="10" spans="1:4" ht="33.9" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>87</v>
       </c>
@@ -8594,7 +8594,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="12" spans="1:4" ht="33.9" customHeight="1">
       <c r="A12" s="4" t="s">
         <v>250</v>
       </c>
@@ -8610,7 +8610,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="13" spans="1:4" ht="33.9" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>251</v>
       </c>
@@ -8626,7 +8626,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="14" spans="1:4" ht="33.9" customHeight="1">
       <c r="A14" s="4" t="s">
         <v>91</v>
       </c>
@@ -8641,7 +8641,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="15" spans="1:4" ht="33.9" customHeight="1">
       <c r="A15" s="4" t="s">
         <v>93</v>
       </c>
@@ -8657,7 +8657,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="16" spans="1:4" ht="33.9" customHeight="1">
       <c r="A16" s="4" t="s">
         <v>94</v>
       </c>
@@ -8673,7 +8673,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="17" spans="1:4" ht="33.9" customHeight="1">
       <c r="A17" s="4" t="s">
         <v>96</v>
       </c>
@@ -8689,7 +8689,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="18" spans="1:4" ht="33.9" customHeight="1">
       <c r="A18" s="4" t="s">
         <v>98</v>
       </c>
@@ -8705,7 +8705,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="19" spans="1:4" ht="33.9" customHeight="1">
       <c r="A19" s="4" t="s">
         <v>100</v>
       </c>
@@ -8753,7 +8753,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="22" spans="1:4" ht="33.9" customHeight="1">
       <c r="A22" s="4" t="s">
         <v>102</v>
       </c>
@@ -8769,7 +8769,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="23" spans="1:4" ht="33.9" customHeight="1">
       <c r="A23" s="4" t="s">
         <v>104</v>
       </c>
@@ -8785,7 +8785,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="24" spans="1:4" ht="33.9" customHeight="1">
       <c r="A24" s="4" t="s">
         <v>105</v>
       </c>
@@ -8801,7 +8801,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="25" spans="1:4" ht="33.9" customHeight="1">
       <c r="A25" s="4" t="s">
         <v>107</v>
       </c>
@@ -8817,7 +8817,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="26" spans="1:4" ht="33.9" customHeight="1">
       <c r="A26" s="16" t="s">
         <v>109</v>
       </c>
@@ -8833,7 +8833,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="27" spans="1:4" ht="33.9" customHeight="1">
       <c r="A27" s="4" t="s">
         <v>111</v>
       </c>
@@ -8849,7 +8849,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="28" spans="1:4" ht="33.9" customHeight="1">
       <c r="A28" s="4" t="s">
         <v>113</v>
       </c>
@@ -8865,7 +8865,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="29" spans="1:4" ht="33.9" customHeight="1">
       <c r="A29" s="4" t="s">
         <v>115</v>
       </c>
@@ -8881,7 +8881,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="30" spans="1:4" ht="33.9" customHeight="1">
       <c r="A30" s="4" t="s">
         <v>117</v>
       </c>
@@ -8897,7 +8897,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="33.950000000000003" customHeight="1">
+    <row r="31" spans="1:4" ht="33.9" customHeight="1">
       <c r="A31" s="4" t="s">
         <v>119</v>
       </c>
@@ -8980,7 +8980,7 @@
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
   <dimension ref="A1:D31"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -8988,30 +8988,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26.1" customHeight="1">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="42" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="42" t="s">
         <v>121</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="C1" s="42" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="D1" s="42" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="36" customHeight="1">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="43" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="39" t="s">
         <v>122</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="39" t="s">
         <v>122</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="40" t="s">
         <v>122</v>
       </c>
     </row>
@@ -9029,7 +9029,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="45.95" customHeight="1">
+    <row r="4" spans="1:4" ht="45.9" customHeight="1">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -9043,7 +9043,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="45.95" customHeight="1">
+    <row r="5" spans="1:4" ht="45.9" customHeight="1">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -9057,7 +9057,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="45.95" customHeight="1">
+    <row r="6" spans="1:4" ht="45.9" customHeight="1">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -9071,7 +9071,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="45.95" customHeight="1">
+    <row r="7" spans="1:4" ht="45.9" customHeight="1">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -9085,7 +9085,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="45.95" customHeight="1">
+    <row r="8" spans="1:4" ht="45.9" customHeight="1">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -9099,7 +9099,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="45.95" customHeight="1">
+    <row r="9" spans="1:4" ht="45.9" customHeight="1">
       <c r="A9" s="12">
         <v>6</v>
       </c>
@@ -9113,7 +9113,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="45.95" customHeight="1">
+    <row r="10" spans="1:4" ht="45.9" customHeight="1">
       <c r="A10" s="12">
         <v>7</v>
       </c>
@@ -9127,7 +9127,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="45.95" customHeight="1">
+    <row r="11" spans="1:4" ht="45.9" customHeight="1">
       <c r="A11" s="12">
         <v>8</v>
       </c>
@@ -9141,7 +9141,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="45.95" customHeight="1">
+    <row r="12" spans="1:4" ht="45.9" customHeight="1">
       <c r="A12" s="12">
         <v>9</v>
       </c>
@@ -9155,7 +9155,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="45.95" customHeight="1">
+    <row r="13" spans="1:4" ht="45.9" customHeight="1">
       <c r="A13" s="12">
         <v>10</v>
       </c>
@@ -9169,7 +9169,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="45.95" customHeight="1">
+    <row r="14" spans="1:4" ht="45.9" customHeight="1">
       <c r="A14" s="12">
         <v>11</v>
       </c>
@@ -9183,7 +9183,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="45.95" customHeight="1">
+    <row r="15" spans="1:4" ht="45.9" customHeight="1">
       <c r="A15" s="12">
         <v>12</v>
       </c>
@@ -9197,7 +9197,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="45.95" customHeight="1">
+    <row r="16" spans="1:4" ht="45.9" customHeight="1">
       <c r="A16" s="12">
         <v>13</v>
       </c>
@@ -9211,7 +9211,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="45.95" customHeight="1">
+    <row r="17" spans="1:4" ht="45.9" customHeight="1">
       <c r="A17" s="12">
         <v>14</v>
       </c>
@@ -9225,7 +9225,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="45.95" customHeight="1">
+    <row r="18" spans="1:4" ht="45.9" customHeight="1">
       <c r="A18" s="12">
         <v>15</v>
       </c>
@@ -9239,7 +9239,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="45.95" customHeight="1">
+    <row r="19" spans="1:4" ht="45.9" customHeight="1">
       <c r="A19" s="12">
         <v>16</v>
       </c>
@@ -9253,7 +9253,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="45.95" customHeight="1">
+    <row r="20" spans="1:4" ht="45.9" customHeight="1">
       <c r="A20" s="12">
         <v>17</v>
       </c>
@@ -9267,7 +9267,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="45.95" customHeight="1">
+    <row r="21" spans="1:4" ht="45.9" customHeight="1">
       <c r="A21" s="12">
         <v>18</v>
       </c>
@@ -9281,7 +9281,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="45.95" customHeight="1">
+    <row r="22" spans="1:4" ht="45.9" customHeight="1">
       <c r="A22" s="12">
         <v>19</v>
       </c>
@@ -9295,7 +9295,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="45.95" customHeight="1">
+    <row r="23" spans="1:4" ht="45.9" customHeight="1">
       <c r="A23" s="12">
         <v>20</v>
       </c>
@@ -9309,7 +9309,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="45.95" customHeight="1">
+    <row r="24" spans="1:4" ht="45.9" customHeight="1">
       <c r="A24" s="12">
         <v>21</v>
       </c>
@@ -9323,7 +9323,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="45.95" customHeight="1">
+    <row r="25" spans="1:4" ht="45.9" customHeight="1">
       <c r="A25" s="12">
         <v>22</v>
       </c>
@@ -9337,7 +9337,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="45.95" customHeight="1">
+    <row r="26" spans="1:4" ht="45.9" customHeight="1">
       <c r="A26" s="12">
         <v>23</v>
       </c>
@@ -9396,9 +9396,9 @@
     <tabColor rgb="FFFFD966"/>
   </sheetPr>
   <dimension ref="A1:AH220"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="23.625" customWidth="1"/>
+    <col min="1" max="1" width="23.59765625" customWidth="1"/>
     <col min="2" max="2" width="3" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="3" customWidth="1"/>
@@ -9417,55 +9417,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="26.1" customHeight="1">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="C1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="D1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="E1" s="46" t="s">
+      <c r="E1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="F1" s="46" t="s">
+      <c r="F1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="G1" s="46" t="s">
+      <c r="G1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="H1" s="46" t="s">
+      <c r="H1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="I1" s="46" t="s">
+      <c r="I1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="J1" s="46" t="s">
+      <c r="J1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="K1" s="46" t="s">
+      <c r="K1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="L1" s="46" t="s">
+      <c r="L1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="M1" s="46" t="s">
+      <c r="M1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="N1" s="46" t="s">
+      <c r="N1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="O1" s="46" t="s">
+      <c r="O1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="P1" s="46" t="s">
+      <c r="P1" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="Q1" s="46" t="s">
+      <c r="Q1" s="42" t="s">
         <v>189</v>
       </c>
       <c r="R1" s="1"/>
@@ -9487,55 +9487,55 @@
       <c r="AH1" s="1"/>
     </row>
     <row r="2" spans="1:34">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="43" t="s">
         <v>258</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="D2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="E2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="F2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="G2" s="28" t="s">
+      <c r="G2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="H2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="I2" s="28" t="s">
+      <c r="I2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="J2" s="28" t="s">
+      <c r="J2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="K2" s="28" t="s">
+      <c r="K2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="L2" s="28" t="s">
+      <c r="L2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="M2" s="28" t="s">
+      <c r="M2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="N2" s="28" t="s">
+      <c r="N2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="O2" s="28" t="s">
+      <c r="O2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="P2" s="28" t="s">
+      <c r="P2" s="39" t="s">
         <v>190</v>
       </c>
-      <c r="Q2" s="29" t="s">
+      <c r="Q2" s="40" t="s">
         <v>190</v>
       </c>
       <c r="R2" s="1"/>
@@ -9592,7 +9592,7 @@
       <c r="AG3" s="1"/>
       <c r="AH3" s="1"/>
     </row>
-    <row r="4" spans="1:34" ht="33.75">
+    <row r="4" spans="1:34" ht="30.6">
       <c r="A4" s="2" t="s">
         <v>191</v>
       </c>
@@ -9780,7 +9780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:34" ht="24">
+    <row r="6" spans="1:34">
       <c r="A6" s="3" t="s">
         <v>260</v>
       </c>
@@ -20836,19 +20836,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100293B981485C9E24DAE651C97D9FBC267" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="73cbee31f6114801cea13732a9ec5387">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="32f33a6e-f018-4796-a6d6-b8c30f0661e9" xmlns:ns3="59ec22bb-74c1-4c3c-af96-122e757b18d2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cc47ff3526632fc7ff348bab4cf07ac" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100293B981485C9E24DAE651C97D9FBC267" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="81e1889baf096e0f1fabc7e628f510b3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="32f33a6e-f018-4796-a6d6-b8c30f0661e9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4b8b816b6954550eb9ea5c593f5cc868" ns2:_="">
     <xsd:import namespace="32f33a6e-f018-4796-a6d6-b8c30f0661e9"/>
-    <xsd:import namespace="59ec22bb-74c1-4c3c-af96-122e757b18d2"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -20858,11 +20854,6 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -20887,43 +20878,6 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="15" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1374c586-51ca-419d-b13a-551147e70874" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="59ec22bb-74c1-4c3c-af96-122e757b18d2" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="16" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{281605ea-d3cc-4310-8c97-aa0e64c9f496}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="59ec22bb-74c1-4c3c-af96-122e757b18d2">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -21026,29 +20980,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="59ec22bb-74c1-4c3c-af96-122e757b18d2" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="32f33a6e-f018-4796-a6d6-b8c30f0661e9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F3F2EB8-DCCD-4569-954D-B034AE82AEB7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{914E18AF-F02E-4042-A16E-8C878EAF693C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59DB138D-8FFF-4EE2-8AA3-13E9CDEF95DB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -21062,4 +21002,30 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CBB2B41-339F-4E9A-AD66-348B65F05334}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="32f33a6e-f018-4796-a6d6-b8c30f0661e9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F3F2EB8-DCCD-4569-954D-B034AE82AEB7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>